<commit_message>
Added relevant files for pricing in workers comp
</commit_message>
<xml_diff>
--- a/srcsc-2026-interest-and-inflation.xlsx
+++ b/srcsc-2026-interest-and-inflation.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="M:\Research\Practice Research\ERM\ERM154-Case Study Challenge\SRCSC 2026\FinalReview\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/atharvamane/Downloads/UNI/ACTL4001/SOA_2026_Case_Study_Materials/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20312715-2B27-4B9E-B84C-7C53F915ED6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5DC96A6-2198-BB4B-99CD-9B5E82C5293C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="810" windowWidth="29040" windowHeight="15720" xr2:uid="{84DBB47E-9408-45F0-9F51-7EAE26B9D89D}"/>
+    <workbookView xWindow="0" yWindow="620" windowWidth="28800" windowHeight="15920" xr2:uid="{84DBB47E-9408-45F0-9F51-7EAE26B9D89D}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -126,33 +126,28 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -376,415 +371,440 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E75FF5A8-7C3D-4731-A799-66F5F2713F93}">
-  <dimension ref="A1:P18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:P24"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.875" style="3" customWidth="1"/>
-    <col min="2" max="2" width="10.5" style="3" customWidth="1"/>
-    <col min="3" max="3" width="16.5" style="3" customWidth="1"/>
-    <col min="4" max="5" width="16.625" style="3" customWidth="1"/>
-    <col min="6" max="16384" width="9" style="1"/>
+    <col min="1" max="1" width="10.83203125" style="2" customWidth="1"/>
+    <col min="2" max="2" width="10.5" style="2" customWidth="1"/>
+    <col min="3" max="3" width="16.5" style="2" customWidth="1"/>
+    <col min="4" max="5" width="16.6640625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
+    <row r="1" spans="1:16" ht="19" x14ac:dyDescent="0.25">
+      <c r="A1" s="7" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:16" s="10" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="11"/>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-    </row>
-    <row r="3" spans="1:16" ht="30" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A2" s="8"/>
+    </row>
+    <row r="3" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+      <c r="A3" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="7" t="s">
+      <c r="C3" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="D3" s="7" t="s">
+      <c r="D3" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="7" t="s">
+      <c r="E3" s="6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A4" s="3">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A4" s="2">
         <v>2160</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="3">
         <v>3.7694526796428575E-2</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="4">
         <v>1.5175498082191765E-3</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="4">
         <v>2.4138414842191764E-3</v>
       </c>
-      <c r="E4" s="5">
+      <c r="E4" s="4">
         <v>3.1124085634359179E-2</v>
       </c>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="M4" s="2"/>
-      <c r="N4" s="2"/>
-      <c r="O4" s="2"/>
-      <c r="P4" s="2"/>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A5" s="3">
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
+      <c r="I4" s="1"/>
+      <c r="J4" s="1"/>
+      <c r="M4" s="1"/>
+      <c r="N4" s="1"/>
+      <c r="O4" s="1"/>
+      <c r="P4" s="1"/>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A5" s="2">
         <v>2161</v>
       </c>
-      <c r="B5" s="4">
+      <c r="B5" s="3">
         <v>2.3173022985428574E-2</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="4">
         <v>1.9996170491803225E-3</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="4">
         <v>2.3921361189803221E-3</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="4">
         <v>2.076300661018032E-2</v>
       </c>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-      <c r="M5" s="2"/>
-      <c r="N5" s="2"/>
-      <c r="O5" s="2"/>
-      <c r="P5" s="2"/>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A6" s="3">
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
+      <c r="J5" s="1"/>
+      <c r="M5" s="1"/>
+      <c r="N5" s="1"/>
+      <c r="O5" s="1"/>
+      <c r="P5" s="1"/>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A6" s="2">
         <v>2162</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B6" s="3">
         <v>1.4768714532000004E-2</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C6" s="4">
         <v>1.6286848000000016E-3</v>
       </c>
-      <c r="D6" s="5">
+      <c r="D6" s="4">
         <v>1.9298700931000016E-3</v>
       </c>
-      <c r="E6" s="5">
+      <c r="E6" s="4">
         <v>2.7251167612330006E-2</v>
       </c>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
-      <c r="M6" s="2"/>
-      <c r="N6" s="2"/>
-      <c r="O6" s="2"/>
-      <c r="P6" s="2"/>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A7" s="3">
+      <c r="G6" s="1"/>
+      <c r="H6" s="1"/>
+      <c r="I6" s="1"/>
+      <c r="J6" s="1"/>
+      <c r="M6" s="1"/>
+      <c r="N6" s="1"/>
+      <c r="O6" s="1"/>
+      <c r="P6" s="1"/>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A7" s="2">
         <v>2163</v>
       </c>
-      <c r="B7" s="4">
+      <c r="B7" s="3">
         <v>1.0826943980142861E-2</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="4">
         <v>1.3475138630136983E-3</v>
       </c>
-      <c r="D7" s="5">
+      <c r="D7" s="4">
         <v>1.7443105410536984E-3</v>
       </c>
-      <c r="E7" s="5">
+      <c r="E7" s="4">
         <v>2.8728069672213696E-2</v>
       </c>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
-      <c r="M7" s="2"/>
-      <c r="N7" s="2"/>
-      <c r="O7" s="2"/>
-      <c r="P7" s="2"/>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A8" s="3">
+      <c r="G7" s="1"/>
+      <c r="H7" s="1"/>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+      <c r="O7" s="1"/>
+      <c r="P7" s="1"/>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A8" s="2">
         <v>2164</v>
       </c>
-      <c r="B8" s="4">
+      <c r="B8" s="3">
         <v>2.161934595000001E-3</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C8" s="4">
         <v>1.8932383123287657E-3</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D8" s="4">
         <v>4.0306069286487655E-3</v>
       </c>
-      <c r="E8" s="5">
+      <c r="E8" s="4">
         <v>2.4318066163208765E-2</v>
       </c>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="M8" s="2"/>
-      <c r="N8" s="2"/>
-      <c r="O8" s="2"/>
-      <c r="P8" s="2"/>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A9" s="3">
+      <c r="G8" s="1"/>
+      <c r="H8" s="1"/>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1"/>
+      <c r="M8" s="1"/>
+      <c r="N8" s="1"/>
+      <c r="O8" s="1"/>
+      <c r="P8" s="1"/>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A9" s="2">
         <v>2165</v>
       </c>
-      <c r="B9" s="4">
+      <c r="B9" s="3">
         <v>7.0673327228571456E-3</v>
       </c>
-      <c r="C9" s="5">
+      <c r="C9" s="4">
         <v>4.808207081967217E-3</v>
       </c>
-      <c r="D9" s="5">
+      <c r="D9" s="4">
         <v>7.1996646525272169E-3</v>
       </c>
-      <c r="E9" s="5">
+      <c r="E9" s="4">
         <v>2.0919444851967218E-2</v>
       </c>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
-      <c r="M9" s="2"/>
-      <c r="N9" s="2"/>
-      <c r="O9" s="2"/>
-      <c r="P9" s="2"/>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A10" s="3">
+      <c r="G9" s="1"/>
+      <c r="H9" s="1"/>
+      <c r="I9" s="1"/>
+      <c r="J9" s="1"/>
+      <c r="M9" s="1"/>
+      <c r="N9" s="1"/>
+      <c r="O9" s="1"/>
+      <c r="P9" s="1"/>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A10" s="2">
         <v>2166</v>
       </c>
-      <c r="B10" s="4">
+      <c r="B10" s="3">
         <v>1.5508568856857145E-2</v>
       </c>
-      <c r="C10" s="5">
+      <c r="C10" s="4">
         <v>1.2019182369146045E-2</v>
       </c>
-      <c r="D10" s="5">
+      <c r="D10" s="4">
         <v>1.4152419484316047E-2</v>
       </c>
-      <c r="E10" s="5">
+      <c r="E10" s="4">
         <v>2.7045913723146044E-2</v>
       </c>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="2"/>
-      <c r="J10" s="2"/>
-      <c r="M10" s="2"/>
-      <c r="N10" s="2"/>
-      <c r="O10" s="2"/>
-      <c r="P10" s="2"/>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A11" s="3">
+      <c r="G10" s="1"/>
+      <c r="H10" s="1"/>
+      <c r="I10" s="1"/>
+      <c r="J10" s="1"/>
+      <c r="M10" s="1"/>
+      <c r="N10" s="1"/>
+      <c r="O10" s="1"/>
+      <c r="P10" s="1"/>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A11" s="2">
         <v>2167</v>
       </c>
-      <c r="B11" s="4">
+      <c r="B11" s="3">
         <v>2.1555430738285718E-2</v>
       </c>
-      <c r="C11" s="5">
+      <c r="C11" s="4">
         <v>2.0303170424242446E-2</v>
       </c>
-      <c r="D11" s="5">
+      <c r="D11" s="4">
         <v>2.1799728471742445E-2</v>
       </c>
-      <c r="E11" s="5">
+      <c r="E11" s="4">
         <v>3.2582581474742446E-2</v>
       </c>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2"/>
-      <c r="M11" s="2"/>
-      <c r="N11" s="2"/>
-      <c r="O11" s="2"/>
-      <c r="P11" s="2"/>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A12" s="3">
+      <c r="G11" s="1"/>
+      <c r="H11" s="1"/>
+      <c r="I11" s="1"/>
+      <c r="J11" s="1"/>
+      <c r="M11" s="1"/>
+      <c r="N11" s="1"/>
+      <c r="O11" s="1"/>
+      <c r="P11" s="1"/>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A12" s="2">
         <v>2168</v>
       </c>
-      <c r="B12" s="4">
+      <c r="B12" s="3">
         <v>1.8084746500000002E-2</v>
       </c>
-      <c r="C12" s="5">
+      <c r="C12" s="4">
         <v>2.4190284111553745E-2</v>
       </c>
-      <c r="D12" s="5">
+      <c r="D12" s="4">
         <v>2.3010827374513744E-2</v>
       </c>
-      <c r="E12" s="5">
+      <c r="E12" s="4">
         <v>2.3993532789553747E-2</v>
       </c>
-      <c r="G12" s="2"/>
-      <c r="H12" s="2"/>
-      <c r="I12" s="2"/>
-      <c r="J12" s="2"/>
-      <c r="M12" s="2"/>
-      <c r="N12" s="2"/>
-      <c r="O12" s="2"/>
-      <c r="P12" s="2"/>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A13" s="3">
+      <c r="G12" s="1"/>
+      <c r="H12" s="1"/>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1"/>
+      <c r="M12" s="1"/>
+      <c r="N12" s="1"/>
+      <c r="O12" s="1"/>
+      <c r="P12" s="1"/>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A13" s="2">
         <v>2169</v>
       </c>
-      <c r="B13" s="4">
+      <c r="B13" s="3">
         <v>7.3377818021428589E-3</v>
       </c>
-      <c r="C13" s="5">
+      <c r="C13" s="4">
         <v>4.3032553359683865E-3</v>
       </c>
-      <c r="D13" s="5">
+      <c r="D13" s="4">
         <v>4.3032553359683865E-3</v>
       </c>
-      <c r="E13" s="5">
+      <c r="E13" s="4">
         <v>9.5032553359683872E-3</v>
       </c>
-      <c r="G13" s="2"/>
-      <c r="H13" s="2"/>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2"/>
-      <c r="M13" s="2"/>
-      <c r="N13" s="2"/>
-      <c r="O13" s="2"/>
-      <c r="P13" s="2"/>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A14" s="3">
+      <c r="G13" s="1"/>
+      <c r="H13" s="1"/>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
+      <c r="M13" s="1"/>
+      <c r="N13" s="1"/>
+      <c r="O13" s="1"/>
+      <c r="P13" s="1"/>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A14" s="2">
         <v>2170</v>
       </c>
-      <c r="B14" s="4">
+      <c r="B14" s="3">
         <v>2.9389208455999998E-2</v>
       </c>
-      <c r="C14" s="5">
+      <c r="C14" s="4">
         <v>1.2531088888888848E-3</v>
       </c>
-      <c r="D14" s="5">
+      <c r="D14" s="4">
         <v>1.4531088888888849E-3</v>
       </c>
-      <c r="E14" s="5">
+      <c r="E14" s="4">
         <v>1.4953108888888884E-2</v>
       </c>
-      <c r="G14" s="2"/>
-      <c r="H14" s="2"/>
-      <c r="I14" s="2"/>
-      <c r="J14" s="2"/>
-      <c r="M14" s="2"/>
-      <c r="N14" s="2"/>
-      <c r="O14" s="2"/>
-      <c r="P14" s="2"/>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A15" s="3">
+      <c r="G14" s="1"/>
+      <c r="H14" s="1"/>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1"/>
+      <c r="M14" s="1"/>
+      <c r="N14" s="1"/>
+      <c r="O14" s="1"/>
+      <c r="P14" s="1"/>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A15" s="2">
         <v>2171</v>
       </c>
-      <c r="B15" s="4">
+      <c r="B15" s="3">
         <v>7.0848661199999996E-2</v>
       </c>
-      <c r="C15" s="5">
+      <c r="C15" s="4">
         <v>1.8250985151999993E-2</v>
       </c>
-      <c r="D15" s="5">
+      <c r="D15" s="4">
         <v>2.9350985151999992E-2</v>
       </c>
-      <c r="E15" s="5">
+      <c r="E15" s="4">
         <v>3.0850985151999993E-2</v>
       </c>
-      <c r="G15" s="2"/>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2"/>
-      <c r="J15" s="2"/>
-      <c r="M15" s="2"/>
-      <c r="N15" s="2"/>
-      <c r="O15" s="2"/>
-      <c r="P15" s="2"/>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A16" s="3">
+      <c r="G15" s="1"/>
+      <c r="H15" s="1"/>
+      <c r="I15" s="1"/>
+      <c r="J15" s="1"/>
+      <c r="M15" s="1"/>
+      <c r="N15" s="1"/>
+      <c r="O15" s="1"/>
+      <c r="P15" s="1"/>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A16" s="2">
         <v>2172</v>
       </c>
-      <c r="B16" s="4">
+      <c r="B16" s="3">
         <v>5.9786544433640419E-2</v>
       </c>
-      <c r="C16" s="5">
+      <c r="C16" s="4">
         <v>5.4047648320000009E-2</v>
       </c>
-      <c r="D16" s="5">
+      <c r="D16" s="4">
         <v>5.454764832000001E-2</v>
       </c>
-      <c r="E16" s="5">
+      <c r="E16" s="4">
         <v>4.3347648320000008E-2</v>
       </c>
-      <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
-      <c r="J16" s="2"/>
-      <c r="M16" s="2"/>
-      <c r="N16" s="2"/>
-      <c r="O16" s="2"/>
-      <c r="P16" s="2"/>
-    </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A17" s="3">
+      <c r="G16" s="1"/>
+      <c r="H16" s="1"/>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1"/>
+      <c r="M16" s="1"/>
+      <c r="N16" s="1"/>
+      <c r="O16" s="1"/>
+      <c r="P16" s="1"/>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A17" s="2">
         <v>2173</v>
       </c>
-      <c r="B17" s="4">
+      <c r="B17" s="3">
         <v>2.7634436430798749E-2</v>
       </c>
-      <c r="C17" s="5">
+      <c r="C17" s="4">
         <v>5.7362710948207142E-2</v>
       </c>
-      <c r="D17" s="5">
+      <c r="D17" s="4">
         <v>5.2762710948207142E-2</v>
       </c>
-      <c r="E17" s="5">
+      <c r="E17" s="4">
         <v>4.7962710948207136E-2</v>
       </c>
-      <c r="G17" s="2"/>
-      <c r="H17" s="2"/>
-      <c r="I17" s="2"/>
-      <c r="J17" s="2"/>
-      <c r="M17" s="2"/>
-      <c r="N17" s="2"/>
-      <c r="O17" s="2"/>
-      <c r="P17" s="2"/>
-    </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A18" s="3">
+      <c r="G17" s="1"/>
+      <c r="H17" s="1"/>
+      <c r="I17" s="1"/>
+      <c r="J17" s="1"/>
+      <c r="M17" s="1"/>
+      <c r="N17" s="1"/>
+      <c r="O17" s="1"/>
+      <c r="P17" s="1"/>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A18" s="2">
         <v>2174</v>
       </c>
-      <c r="B18" s="4">
+      <c r="B18" s="3">
         <v>2.3905736589285704E-2</v>
       </c>
-      <c r="C18" s="5">
+      <c r="C18" s="4">
         <v>5.0506368421052765E-2</v>
       </c>
-      <c r="D18" s="5">
+      <c r="D18" s="4">
         <v>4.7406368421052766E-2</v>
       </c>
-      <c r="E18" s="5">
+      <c r="E18" s="4">
         <v>5.1006368421052765E-2</v>
       </c>
-      <c r="G18" s="2"/>
-      <c r="H18" s="2"/>
-      <c r="I18" s="2"/>
-      <c r="J18" s="2"/>
+      <c r="G18" s="1"/>
+      <c r="H18" s="1"/>
+      <c r="I18" s="1"/>
+      <c r="J18" s="1"/>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A19" s="2">
+        <v>2175</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A20" s="2">
+        <v>2176</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A21" s="2">
+        <v>2177</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A22" s="2">
+        <v>2178</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A23" s="2">
+        <v>2179</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.2">
+      <c r="A24" s="2">
+        <v>2180</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -792,6 +812,25 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="16a415e0-cbd2-494f-bd0b-9ec9526163e9">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100A13D16CE4023BB4BB4110DFC2802C897" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="65b3ef4f2db57c8fd06e10d67e29a91c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="16a415e0-cbd2-494f-bd0b-9ec9526163e9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="368f79d5404671231dfb7196e18a5373" ns2:_="">
     <xsd:import namespace="16a415e0-cbd2-494f-bd0b-9ec9526163e9"/>
@@ -981,33 +1020,38 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="16a415e0-cbd2-494f-bd0b-9ec9526163e9">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F19435BB-84D2-485C-9BB4-65747E4E117C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82E76C6D-4CB6-49CD-887A-00EE2372E5AB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="16a415e0-cbd2-494f-bd0b-9ec9526163e9"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19394A87-9C0F-4429-B344-1F754C914B7C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{19394A87-9C0F-4429-B344-1F754C914B7C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{82E76C6D-4CB6-49CD-887A-00EE2372E5AB}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F19435BB-84D2-485C-9BB4-65747E4E117C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="16a415e0-cbd2-494f-bd0b-9ec9526163e9"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>